<commit_message>
adding feature to detect aircraft involved in a fire and Oil Rigs
</commit_message>
<xml_diff>
--- a/doc/credit_usage.xlsx
+++ b/doc/credit_usage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\lngo\projects\aero-hydra\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621ED89B-215C-4288-B6CF-4EA1D6E32292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE5A232-2605-4805-8163-A9E80F265E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13125" yWindow="1905" windowWidth="26055" windowHeight="17790" xr2:uid="{0EA86F42-7427-4896-83BC-75805D4D4BE4}"/>
+    <workbookView xWindow="12855" yWindow="2925" windowWidth="24270" windowHeight="16890" xr2:uid="{0EA86F42-7427-4896-83BC-75805D4D4BE4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1170,11 +1170,11 @@
       </c>
       <c r="AG4">
         <f t="shared" ref="AG4:AG28" si="0">AD4*$B$4+AE4*$B$5</f>
-        <v>773</v>
+        <v>890</v>
       </c>
       <c r="AH4" s="29">
         <f t="shared" ref="AH4:AH28" si="1">AG4/4000</f>
-        <v>0.19325000000000001</v>
+        <v>0.2225</v>
       </c>
       <c r="AI4" s="20"/>
     </row>
@@ -1183,7 +1183,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="23">
         <v>0</v>
@@ -1194,91 +1194,91 @@
       </c>
       <c r="F5" s="21">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *F$4</f>
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="G5" s="21">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *G$4</f>
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="H5" s="21">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *H$4</f>
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="I5" s="21">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *I$4</f>
-        <v>330</v>
+        <v>360</v>
       </c>
       <c r="J5" s="21">
         <f t="shared" ref="J5:AA20" si="2">$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *J$4</f>
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="K5" s="21">
         <f t="shared" si="2"/>
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="L5" s="21">
         <f t="shared" si="2"/>
-        <v>570</v>
+        <v>600</v>
       </c>
       <c r="M5" s="21">
         <f t="shared" si="2"/>
-        <v>630</v>
+        <v>660</v>
       </c>
       <c r="N5" s="21">
         <f t="shared" si="2"/>
-        <v>690</v>
+        <v>720</v>
       </c>
       <c r="O5" s="21">
         <f t="shared" si="2"/>
-        <v>750</v>
+        <v>780</v>
       </c>
       <c r="P5" s="21">
         <f t="shared" si="2"/>
-        <v>810</v>
+        <v>840</v>
       </c>
       <c r="Q5" s="21">
         <f t="shared" si="2"/>
-        <v>870</v>
+        <v>900</v>
       </c>
       <c r="R5" s="21">
         <f t="shared" si="2"/>
-        <v>930</v>
+        <v>960</v>
       </c>
       <c r="S5" s="21">
         <f t="shared" si="2"/>
-        <v>990</v>
+        <v>1020</v>
       </c>
       <c r="T5" s="21">
         <f t="shared" si="2"/>
-        <v>1290</v>
+        <v>1320</v>
       </c>
       <c r="U5" s="21">
         <f t="shared" ref="U5:V20" si="3">$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *U$4</f>
-        <v>1350</v>
+        <v>1380</v>
       </c>
       <c r="V5" s="22">
         <f t="shared" si="3"/>
-        <v>1410</v>
+        <v>1440</v>
       </c>
       <c r="W5" s="23">
         <f t="shared" si="2"/>
-        <v>1470</v>
+        <v>1500</v>
       </c>
       <c r="X5" s="24">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *X$4</f>
-        <v>1590</v>
+        <v>1620</v>
       </c>
       <c r="Y5" s="21">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *Y$4</f>
-        <v>1890</v>
+        <v>1920</v>
       </c>
       <c r="Z5" s="21">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *Z$4</f>
-        <v>2190</v>
+        <v>2220</v>
       </c>
       <c r="AA5" s="7">
         <f>$B$5*($D5+1)*(60/$B$3) + $B$4*($D5+1)*(60/$B$3) *AA$4</f>
-        <v>2490</v>
+        <v>2520</v>
       </c>
       <c r="AC5" t="s">
         <v>16</v>
@@ -1291,11 +1291,11 @@
       </c>
       <c r="AG5">
         <f>AD5*$B$4+AE5*$B$5</f>
-        <v>1345</v>
+        <v>1644</v>
       </c>
       <c r="AH5" s="29">
         <f t="shared" si="1"/>
-        <v>0.33624999999999999</v>
+        <v>0.41099999999999998</v>
       </c>
       <c r="AI5" s="20">
         <f>AD5/AE5</f>
@@ -1312,91 +1312,91 @@
       </c>
       <c r="F6" s="1">
         <f t="shared" ref="F6:AA28" si="5">$B$5*($D6+1)*(60/$B$3) + $B$4*($D6+1)*(60/$B$3) *F$4</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="G6" s="1">
         <f t="shared" si="5"/>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="5"/>
-        <v>540</v>
+        <v>600</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="5"/>
-        <v>660</v>
+        <v>720</v>
       </c>
       <c r="J6" s="1">
         <f t="shared" si="2"/>
-        <v>900</v>
+        <v>960</v>
       </c>
       <c r="K6" s="1">
         <f t="shared" si="2"/>
-        <v>1020</v>
+        <v>1080</v>
       </c>
       <c r="L6" s="1">
         <f t="shared" si="2"/>
-        <v>1140</v>
+        <v>1200</v>
       </c>
       <c r="M6" s="1">
         <f t="shared" si="2"/>
-        <v>1260</v>
+        <v>1320</v>
       </c>
       <c r="N6" s="1">
         <f t="shared" si="2"/>
-        <v>1380</v>
+        <v>1440</v>
       </c>
       <c r="O6" s="1">
         <f t="shared" si="2"/>
-        <v>1500</v>
+        <v>1560</v>
       </c>
       <c r="P6" s="1">
         <f t="shared" si="2"/>
-        <v>1620</v>
+        <v>1680</v>
       </c>
       <c r="Q6" s="1">
         <f t="shared" si="2"/>
-        <v>1740</v>
+        <v>1800</v>
       </c>
       <c r="R6" s="1">
         <f t="shared" si="2"/>
-        <v>1860</v>
+        <v>1920</v>
       </c>
       <c r="S6" s="1">
         <f t="shared" si="2"/>
-        <v>1980</v>
+        <v>2040</v>
       </c>
       <c r="T6" s="1">
         <f t="shared" ref="T6:V28" si="6">$B$5*($D6+1)*(60/$B$3) + $B$4*($D6+1)*(60/$B$3) *T$4</f>
-        <v>2580</v>
+        <v>2640</v>
       </c>
       <c r="U6" s="1">
         <f t="shared" si="3"/>
-        <v>2700</v>
+        <v>2760</v>
       </c>
       <c r="V6" s="2">
         <f t="shared" si="3"/>
-        <v>2820</v>
+        <v>2880</v>
       </c>
       <c r="W6" s="4">
         <f t="shared" si="2"/>
-        <v>2940</v>
+        <v>3000</v>
       </c>
       <c r="X6" s="3">
         <f t="shared" si="2"/>
-        <v>3180</v>
+        <v>3240</v>
       </c>
       <c r="Y6" s="1">
         <f t="shared" si="2"/>
-        <v>3780</v>
+        <v>3840</v>
       </c>
       <c r="Z6" s="1">
         <f t="shared" si="2"/>
-        <v>4380</v>
+        <v>4440</v>
       </c>
       <c r="AA6" s="9">
         <f t="shared" si="2"/>
-        <v>4980</v>
+        <v>5040</v>
       </c>
       <c r="AC6" t="s">
         <v>13</v>
@@ -1409,11 +1409,11 @@
       </c>
       <c r="AG6">
         <f t="shared" si="0"/>
-        <v>1112</v>
+        <v>1452</v>
       </c>
       <c r="AH6" s="29">
         <f t="shared" si="1"/>
-        <v>0.27800000000000002</v>
+        <v>0.36299999999999999</v>
       </c>
       <c r="AI6" s="20">
         <f t="shared" ref="AI6:AI28" si="7">AD6/AE6</f>
@@ -1430,91 +1430,91 @@
       </c>
       <c r="F7" s="1">
         <f t="shared" si="5"/>
-        <v>450</v>
+        <v>540</v>
       </c>
       <c r="G7" s="1">
         <f t="shared" si="5"/>
-        <v>630</v>
+        <v>720</v>
       </c>
       <c r="H7" s="1">
         <f t="shared" si="5"/>
-        <v>810</v>
+        <v>900</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="5"/>
-        <v>990</v>
+        <v>1080</v>
       </c>
       <c r="J7" s="1">
         <f t="shared" si="2"/>
-        <v>1350</v>
+        <v>1440</v>
       </c>
       <c r="K7" s="1">
         <f t="shared" si="2"/>
-        <v>1530</v>
+        <v>1620</v>
       </c>
       <c r="L7" s="1">
         <f t="shared" si="2"/>
-        <v>1710</v>
+        <v>1800</v>
       </c>
       <c r="M7" s="1">
         <f t="shared" si="2"/>
-        <v>1890</v>
+        <v>1980</v>
       </c>
       <c r="N7" s="1">
         <f t="shared" si="2"/>
-        <v>2070</v>
+        <v>2160</v>
       </c>
       <c r="O7" s="1">
         <f t="shared" si="2"/>
-        <v>2250</v>
+        <v>2340</v>
       </c>
       <c r="P7" s="1">
         <f t="shared" si="2"/>
-        <v>2430</v>
+        <v>2520</v>
       </c>
       <c r="Q7" s="1">
         <f t="shared" si="2"/>
-        <v>2610</v>
+        <v>2700</v>
       </c>
       <c r="R7" s="1">
         <f t="shared" si="2"/>
-        <v>2790</v>
+        <v>2880</v>
       </c>
       <c r="S7" s="1">
         <f t="shared" si="2"/>
-        <v>2970</v>
+        <v>3060</v>
       </c>
       <c r="T7" s="1">
         <f t="shared" si="6"/>
-        <v>3870</v>
+        <v>3960</v>
       </c>
       <c r="U7" s="1">
         <f t="shared" si="3"/>
-        <v>4050</v>
+        <v>4140</v>
       </c>
       <c r="V7" s="2">
         <f t="shared" si="3"/>
-        <v>4230</v>
+        <v>4320</v>
       </c>
       <c r="W7" s="4">
         <f t="shared" si="2"/>
-        <v>4410</v>
+        <v>4500</v>
       </c>
       <c r="X7" s="3">
         <f t="shared" si="2"/>
-        <v>4770</v>
+        <v>4860</v>
       </c>
       <c r="Y7" s="1">
         <f t="shared" si="2"/>
-        <v>5670</v>
+        <v>5760</v>
       </c>
       <c r="Z7" s="1">
         <f t="shared" si="2"/>
-        <v>6570</v>
+        <v>6660</v>
       </c>
       <c r="AA7" s="9">
         <f t="shared" si="2"/>
-        <v>7470</v>
+        <v>7560</v>
       </c>
       <c r="AC7" s="26" t="s">
         <v>17</v>
@@ -1527,11 +1527,11 @@
       </c>
       <c r="AG7">
         <f t="shared" si="0"/>
-        <v>1644</v>
+        <v>1984</v>
       </c>
       <c r="AH7" s="29">
         <f t="shared" si="1"/>
-        <v>0.41099999999999998</v>
+        <v>0.496</v>
       </c>
       <c r="AI7" s="20">
         <f t="shared" si="7"/>
@@ -1548,91 +1548,91 @@
       </c>
       <c r="F8" s="1">
         <f t="shared" si="5"/>
-        <v>600</v>
+        <v>720</v>
       </c>
       <c r="G8" s="1">
         <f t="shared" si="5"/>
-        <v>840</v>
+        <v>960</v>
       </c>
       <c r="H8" s="1">
         <f t="shared" si="5"/>
-        <v>1080</v>
+        <v>1200</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="5"/>
-        <v>1320</v>
+        <v>1440</v>
       </c>
       <c r="J8" s="1">
         <f t="shared" si="2"/>
-        <v>1800</v>
+        <v>1920</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" si="2"/>
-        <v>2040</v>
+        <v>2160</v>
       </c>
       <c r="L8" s="1">
         <f t="shared" si="2"/>
-        <v>2280</v>
+        <v>2400</v>
       </c>
       <c r="M8" s="1">
         <f t="shared" si="2"/>
-        <v>2520</v>
+        <v>2640</v>
       </c>
       <c r="N8" s="1">
         <f t="shared" si="2"/>
-        <v>2760</v>
+        <v>2880</v>
       </c>
       <c r="O8" s="1">
         <f t="shared" si="2"/>
-        <v>3000</v>
+        <v>3120</v>
       </c>
       <c r="P8" s="1">
         <f t="shared" si="2"/>
-        <v>3240</v>
+        <v>3360</v>
       </c>
       <c r="Q8" s="1">
         <f t="shared" si="2"/>
-        <v>3480</v>
+        <v>3600</v>
       </c>
       <c r="R8" s="1">
         <f t="shared" si="2"/>
-        <v>3720</v>
+        <v>3840</v>
       </c>
       <c r="S8" s="1">
         <f t="shared" si="2"/>
-        <v>3960</v>
+        <v>4080</v>
       </c>
       <c r="T8" s="1">
         <f t="shared" si="6"/>
-        <v>5160</v>
+        <v>5280</v>
       </c>
       <c r="U8" s="1">
         <f t="shared" si="3"/>
-        <v>5400</v>
+        <v>5520</v>
       </c>
       <c r="V8" s="2">
         <f t="shared" si="3"/>
-        <v>5640</v>
+        <v>5760</v>
       </c>
       <c r="W8" s="4">
         <f t="shared" si="2"/>
-        <v>5880</v>
+        <v>6000</v>
       </c>
       <c r="X8" s="3">
         <f t="shared" si="2"/>
-        <v>6360</v>
+        <v>6480</v>
       </c>
       <c r="Y8" s="1">
         <f t="shared" si="2"/>
-        <v>7560</v>
+        <v>7680</v>
       </c>
       <c r="Z8" s="1">
         <f t="shared" si="2"/>
-        <v>8760</v>
+        <v>8880</v>
       </c>
       <c r="AA8" s="9">
         <f t="shared" si="2"/>
-        <v>9960</v>
+        <v>10080</v>
       </c>
       <c r="AC8" s="26" t="s">
         <v>18</v>
@@ -1645,11 +1645,11 @@
       </c>
       <c r="AG8">
         <f t="shared" si="0"/>
-        <v>1604</v>
+        <v>1944</v>
       </c>
       <c r="AH8" s="29">
         <f t="shared" si="1"/>
-        <v>0.40100000000000002</v>
+        <v>0.48599999999999999</v>
       </c>
       <c r="AI8" s="20">
         <f t="shared" si="7"/>
@@ -1666,91 +1666,91 @@
       </c>
       <c r="F9" s="1">
         <f t="shared" si="5"/>
-        <v>750</v>
+        <v>900</v>
       </c>
       <c r="G9" s="1">
         <f t="shared" si="5"/>
-        <v>1050</v>
+        <v>1200</v>
       </c>
       <c r="H9" s="1">
         <f t="shared" si="5"/>
-        <v>1350</v>
+        <v>1500</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="5"/>
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="J9" s="1">
         <f t="shared" si="2"/>
-        <v>2250</v>
+        <v>2400</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" si="2"/>
-        <v>2550</v>
+        <v>2700</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="2"/>
-        <v>2850</v>
+        <v>3000</v>
       </c>
       <c r="M9" s="1">
         <f t="shared" si="2"/>
-        <v>3150</v>
+        <v>3300</v>
       </c>
       <c r="N9" s="1">
         <f t="shared" si="2"/>
-        <v>3450</v>
+        <v>3600</v>
       </c>
       <c r="O9" s="1">
         <f t="shared" si="2"/>
-        <v>3750</v>
+        <v>3900</v>
       </c>
       <c r="P9" s="1">
         <f t="shared" si="2"/>
-        <v>4050</v>
+        <v>4200</v>
       </c>
       <c r="Q9" s="1">
         <f t="shared" si="2"/>
-        <v>4350</v>
+        <v>4500</v>
       </c>
       <c r="R9" s="1">
         <f t="shared" si="2"/>
-        <v>4650</v>
+        <v>4800</v>
       </c>
       <c r="S9" s="1">
         <f t="shared" si="2"/>
-        <v>4950</v>
+        <v>5100</v>
       </c>
       <c r="T9" s="1">
         <f t="shared" si="6"/>
-        <v>6450</v>
+        <v>6600</v>
       </c>
       <c r="U9" s="1">
         <f t="shared" si="3"/>
-        <v>6750</v>
+        <v>6900</v>
       </c>
       <c r="V9" s="2">
         <f t="shared" si="3"/>
-        <v>7050</v>
+        <v>7200</v>
       </c>
       <c r="W9" s="4">
         <f t="shared" si="2"/>
-        <v>7350</v>
+        <v>7500</v>
       </c>
       <c r="X9" s="3">
         <f t="shared" si="2"/>
-        <v>7950</v>
+        <v>8100</v>
       </c>
       <c r="Y9" s="1">
         <f t="shared" si="2"/>
-        <v>9450</v>
+        <v>9600</v>
       </c>
       <c r="Z9" s="1">
         <f t="shared" si="2"/>
-        <v>10950</v>
+        <v>11100</v>
       </c>
       <c r="AA9" s="9">
         <f t="shared" si="2"/>
-        <v>12450</v>
+        <v>12600</v>
       </c>
       <c r="AC9" t="s">
         <v>19</v>
@@ -1763,11 +1763,11 @@
       </c>
       <c r="AG9">
         <f t="shared" si="0"/>
-        <v>1498</v>
+        <v>1838</v>
       </c>
       <c r="AH9" s="29">
         <f t="shared" si="1"/>
-        <v>0.3745</v>
+        <v>0.45950000000000002</v>
       </c>
       <c r="AI9" s="20">
         <f t="shared" si="7"/>
@@ -1784,91 +1784,91 @@
       </c>
       <c r="F10" s="1">
         <f t="shared" si="5"/>
-        <v>900</v>
+        <v>1080</v>
       </c>
       <c r="G10" s="1">
         <f t="shared" si="5"/>
-        <v>1260</v>
+        <v>1440</v>
       </c>
       <c r="H10" s="1">
         <f t="shared" si="5"/>
-        <v>1620</v>
+        <v>1800</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="5"/>
-        <v>1980</v>
+        <v>2160</v>
       </c>
       <c r="J10" s="1">
         <f t="shared" si="2"/>
-        <v>2700</v>
+        <v>2880</v>
       </c>
       <c r="K10" s="1">
         <f t="shared" si="2"/>
-        <v>3060</v>
+        <v>3240</v>
       </c>
       <c r="L10" s="1">
         <f t="shared" si="2"/>
-        <v>3420</v>
+        <v>3600</v>
       </c>
       <c r="M10" s="1">
         <f t="shared" si="2"/>
-        <v>3780</v>
+        <v>3960</v>
       </c>
       <c r="N10" s="1">
         <f t="shared" si="2"/>
-        <v>4140</v>
+        <v>4320</v>
       </c>
       <c r="O10" s="1">
         <f t="shared" si="2"/>
-        <v>4500</v>
+        <v>4680</v>
       </c>
       <c r="P10" s="1">
         <f t="shared" si="2"/>
-        <v>4860</v>
+        <v>5040</v>
       </c>
       <c r="Q10" s="1">
         <f t="shared" si="2"/>
-        <v>5220</v>
+        <v>5400</v>
       </c>
       <c r="R10" s="1">
         <f t="shared" si="2"/>
-        <v>5580</v>
+        <v>5760</v>
       </c>
       <c r="S10" s="1">
         <f t="shared" si="2"/>
-        <v>5940</v>
+        <v>6120</v>
       </c>
       <c r="T10" s="1">
         <f t="shared" si="6"/>
-        <v>7740</v>
+        <v>7920</v>
       </c>
       <c r="U10" s="1">
         <f t="shared" si="3"/>
-        <v>8100</v>
+        <v>8280</v>
       </c>
       <c r="V10" s="2">
         <f t="shared" si="3"/>
-        <v>8460</v>
+        <v>8640</v>
       </c>
       <c r="W10" s="4">
         <f t="shared" si="2"/>
-        <v>8820</v>
+        <v>9000</v>
       </c>
       <c r="X10" s="3">
         <f t="shared" si="2"/>
-        <v>9540</v>
+        <v>9720</v>
       </c>
       <c r="Y10" s="1">
         <f t="shared" si="2"/>
-        <v>11340</v>
+        <v>11520</v>
       </c>
       <c r="Z10" s="1">
         <f t="shared" si="2"/>
-        <v>13140</v>
+        <v>13320</v>
       </c>
       <c r="AA10" s="9">
         <f t="shared" si="2"/>
-        <v>14940</v>
+        <v>15120</v>
       </c>
       <c r="AC10" s="27" t="s">
         <v>20</v>
@@ -1882,11 +1882,11 @@
       <c r="AF10" s="27"/>
       <c r="AG10" s="27">
         <f t="shared" si="0"/>
-        <v>2516</v>
+        <v>2856</v>
       </c>
       <c r="AH10" s="30">
         <f t="shared" si="1"/>
-        <v>0.629</v>
+        <v>0.71399999999999997</v>
       </c>
       <c r="AI10" s="28">
         <f t="shared" si="7"/>
@@ -1906,91 +1906,91 @@
       </c>
       <c r="F11" s="1">
         <f t="shared" si="5"/>
-        <v>1050</v>
+        <v>1260</v>
       </c>
       <c r="G11" s="1">
         <f t="shared" si="5"/>
-        <v>1470</v>
+        <v>1680</v>
       </c>
       <c r="H11" s="1">
         <f t="shared" si="5"/>
-        <v>1890</v>
+        <v>2100</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="5"/>
-        <v>2310</v>
+        <v>2520</v>
       </c>
       <c r="J11" s="1">
         <f t="shared" si="2"/>
-        <v>3150</v>
+        <v>3360</v>
       </c>
       <c r="K11" s="1">
         <f t="shared" si="2"/>
-        <v>3570</v>
+        <v>3780</v>
       </c>
       <c r="L11" s="1">
         <f t="shared" si="2"/>
-        <v>3990</v>
+        <v>4200</v>
       </c>
       <c r="M11" s="1">
         <f t="shared" si="2"/>
-        <v>4410</v>
+        <v>4620</v>
       </c>
       <c r="N11" s="1">
         <f t="shared" si="2"/>
-        <v>4830</v>
+        <v>5040</v>
       </c>
       <c r="O11" s="1">
         <f t="shared" si="2"/>
-        <v>5250</v>
+        <v>5460</v>
       </c>
       <c r="P11" s="1">
         <f t="shared" si="2"/>
-        <v>5670</v>
+        <v>5880</v>
       </c>
       <c r="Q11" s="1">
         <f t="shared" si="2"/>
-        <v>6090</v>
+        <v>6300</v>
       </c>
       <c r="R11" s="1">
         <f t="shared" si="2"/>
-        <v>6510</v>
+        <v>6720</v>
       </c>
       <c r="S11" s="1">
         <f t="shared" si="2"/>
-        <v>6930</v>
+        <v>7140</v>
       </c>
       <c r="T11" s="1">
         <f t="shared" si="6"/>
-        <v>9030</v>
+        <v>9240</v>
       </c>
       <c r="U11" s="1">
         <f t="shared" si="3"/>
-        <v>9450</v>
+        <v>9660</v>
       </c>
       <c r="V11" s="2">
         <f t="shared" si="3"/>
-        <v>9870</v>
+        <v>10080</v>
       </c>
       <c r="W11" s="4">
         <f t="shared" si="2"/>
-        <v>10290</v>
+        <v>10500</v>
       </c>
       <c r="X11" s="3">
         <f t="shared" si="2"/>
-        <v>11130</v>
+        <v>11340</v>
       </c>
       <c r="Y11" s="1">
         <f t="shared" si="2"/>
-        <v>13230</v>
+        <v>13440</v>
       </c>
       <c r="Z11" s="1">
         <f t="shared" si="2"/>
-        <v>15330</v>
+        <v>15540</v>
       </c>
       <c r="AA11" s="9">
         <f t="shared" si="2"/>
-        <v>17430</v>
+        <v>17640</v>
       </c>
       <c r="AC11" s="31" t="s">
         <v>22</v>
@@ -2006,11 +2006,11 @@
       </c>
       <c r="AG11" s="31">
         <f t="shared" si="0"/>
-        <v>4259</v>
+        <v>4834</v>
       </c>
       <c r="AH11" s="32">
         <f t="shared" si="1"/>
-        <v>1.0647500000000001</v>
+        <v>1.2084999999999999</v>
       </c>
       <c r="AI11" s="33">
         <f>(AD11-AF11)/AE11</f>
@@ -2030,91 +2030,91 @@
       </c>
       <c r="F12" s="1">
         <f t="shared" si="5"/>
-        <v>1200</v>
+        <v>1440</v>
       </c>
       <c r="G12" s="1">
         <f t="shared" si="5"/>
-        <v>1680</v>
+        <v>1920</v>
       </c>
       <c r="H12" s="1">
         <f t="shared" si="5"/>
-        <v>2160</v>
+        <v>2400</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="5"/>
-        <v>2640</v>
+        <v>2880</v>
       </c>
       <c r="J12" s="1">
         <f t="shared" si="2"/>
-        <v>3600</v>
+        <v>3840</v>
       </c>
       <c r="K12" s="1">
         <f t="shared" si="2"/>
-        <v>4080</v>
+        <v>4320</v>
       </c>
       <c r="L12" s="1">
         <f t="shared" si="2"/>
-        <v>4560</v>
+        <v>4800</v>
       </c>
       <c r="M12" s="1">
         <f t="shared" si="2"/>
-        <v>5040</v>
+        <v>5280</v>
       </c>
       <c r="N12" s="1">
         <f t="shared" si="2"/>
-        <v>5520</v>
+        <v>5760</v>
       </c>
       <c r="O12" s="1">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>6240</v>
       </c>
       <c r="P12" s="1">
         <f t="shared" si="2"/>
-        <v>6480</v>
+        <v>6720</v>
       </c>
       <c r="Q12" s="1">
         <f t="shared" si="2"/>
-        <v>6960</v>
+        <v>7200</v>
       </c>
       <c r="R12" s="1">
         <f t="shared" si="2"/>
-        <v>7440</v>
+        <v>7680</v>
       </c>
       <c r="S12" s="1">
         <f t="shared" si="2"/>
-        <v>7920</v>
+        <v>8160</v>
       </c>
       <c r="T12" s="1">
         <f t="shared" si="6"/>
-        <v>10320</v>
+        <v>10560</v>
       </c>
       <c r="U12" s="1">
         <f t="shared" si="3"/>
-        <v>10800</v>
+        <v>11040</v>
       </c>
       <c r="V12" s="2">
         <f t="shared" si="3"/>
-        <v>11280</v>
+        <v>11520</v>
       </c>
       <c r="W12" s="4">
         <f t="shared" si="2"/>
-        <v>11760</v>
+        <v>12000</v>
       </c>
       <c r="X12" s="3">
         <f t="shared" si="2"/>
-        <v>12720</v>
+        <v>12960</v>
       </c>
       <c r="Y12" s="1">
         <f t="shared" si="2"/>
-        <v>15120</v>
+        <v>15360</v>
       </c>
       <c r="Z12" s="1">
         <f t="shared" si="2"/>
-        <v>17520</v>
+        <v>17760</v>
       </c>
       <c r="AA12" s="9">
         <f t="shared" si="2"/>
-        <v>19920</v>
+        <v>20160</v>
       </c>
       <c r="AC12" t="s">
         <v>25</v>
@@ -2127,11 +2127,11 @@
       </c>
       <c r="AG12">
         <f t="shared" si="0"/>
-        <v>2500</v>
+        <v>3010</v>
       </c>
       <c r="AH12" s="29">
         <f t="shared" si="1"/>
-        <v>0.625</v>
+        <v>0.75249999999999995</v>
       </c>
       <c r="AI12" s="20">
         <f t="shared" si="7"/>
@@ -2148,91 +2148,91 @@
       </c>
       <c r="F13" s="1">
         <f t="shared" si="5"/>
-        <v>1350</v>
+        <v>1620</v>
       </c>
       <c r="G13" s="1">
         <f t="shared" si="5"/>
-        <v>1890</v>
+        <v>2160</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="5"/>
-        <v>2430</v>
+        <v>2700</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="5"/>
-        <v>2970</v>
+        <v>3240</v>
       </c>
       <c r="J13" s="1">
         <f t="shared" si="2"/>
-        <v>4050</v>
+        <v>4320</v>
       </c>
       <c r="K13" s="1">
         <f t="shared" si="2"/>
-        <v>4590</v>
+        <v>4860</v>
       </c>
       <c r="L13" s="1">
         <f t="shared" si="2"/>
-        <v>5130</v>
+        <v>5400</v>
       </c>
       <c r="M13" s="1">
         <f t="shared" si="2"/>
-        <v>5670</v>
+        <v>5940</v>
       </c>
       <c r="N13" s="1">
         <f t="shared" si="2"/>
-        <v>6210</v>
+        <v>6480</v>
       </c>
       <c r="O13" s="1">
         <f t="shared" si="2"/>
-        <v>6750</v>
+        <v>7020</v>
       </c>
       <c r="P13" s="1">
         <f t="shared" si="2"/>
-        <v>7290</v>
+        <v>7560</v>
       </c>
       <c r="Q13" s="1">
         <f t="shared" si="2"/>
-        <v>7830</v>
+        <v>8100</v>
       </c>
       <c r="R13" s="1">
         <f t="shared" si="2"/>
-        <v>8370</v>
+        <v>8640</v>
       </c>
       <c r="S13" s="1">
         <f t="shared" si="2"/>
-        <v>8910</v>
+        <v>9180</v>
       </c>
       <c r="T13" s="1">
         <f t="shared" si="6"/>
-        <v>11610</v>
+        <v>11880</v>
       </c>
       <c r="U13" s="1">
         <f t="shared" si="3"/>
-        <v>12150</v>
+        <v>12420</v>
       </c>
       <c r="V13" s="2">
         <f t="shared" si="3"/>
-        <v>12690</v>
+        <v>12960</v>
       </c>
       <c r="W13" s="4">
         <f t="shared" si="2"/>
-        <v>13230</v>
+        <v>13500</v>
       </c>
       <c r="X13" s="3">
         <f t="shared" si="2"/>
-        <v>14310</v>
+        <v>14580</v>
       </c>
       <c r="Y13" s="1">
         <f t="shared" si="2"/>
-        <v>17010</v>
+        <v>17280</v>
       </c>
       <c r="Z13" s="1">
         <f t="shared" si="2"/>
-        <v>19710</v>
+        <v>19980</v>
       </c>
       <c r="AA13" s="9">
         <f t="shared" si="2"/>
-        <v>22410</v>
+        <v>22680</v>
       </c>
       <c r="AC13" t="s">
         <v>26</v>
@@ -2245,11 +2245,11 @@
       </c>
       <c r="AG13">
         <f t="shared" si="0"/>
-        <v>2878</v>
+        <v>3388</v>
       </c>
       <c r="AH13" s="29">
         <f t="shared" si="1"/>
-        <v>0.71950000000000003</v>
+        <v>0.84699999999999998</v>
       </c>
       <c r="AI13" s="20">
         <f t="shared" si="7"/>
@@ -2266,91 +2266,91 @@
       </c>
       <c r="F14" s="1">
         <f t="shared" si="5"/>
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="G14" s="1">
         <f t="shared" si="5"/>
-        <v>2100</v>
+        <v>2400</v>
       </c>
       <c r="H14" s="1">
         <f t="shared" si="5"/>
-        <v>2700</v>
+        <v>3000</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="5"/>
-        <v>3300</v>
+        <v>3600</v>
       </c>
       <c r="J14" s="1">
         <f t="shared" si="2"/>
-        <v>4500</v>
+        <v>4800</v>
       </c>
       <c r="K14" s="1">
         <f t="shared" si="2"/>
-        <v>5100</v>
+        <v>5400</v>
       </c>
       <c r="L14" s="1">
         <f t="shared" si="2"/>
-        <v>5700</v>
+        <v>6000</v>
       </c>
       <c r="M14" s="1">
         <f t="shared" si="2"/>
-        <v>6300</v>
+        <v>6600</v>
       </c>
       <c r="N14" s="1">
         <f t="shared" si="2"/>
-        <v>6900</v>
+        <v>7200</v>
       </c>
       <c r="O14" s="1">
         <f t="shared" si="2"/>
-        <v>7500</v>
+        <v>7800</v>
       </c>
       <c r="P14" s="1">
         <f t="shared" si="2"/>
-        <v>8100</v>
+        <v>8400</v>
       </c>
       <c r="Q14" s="1">
         <f t="shared" si="2"/>
-        <v>8700</v>
+        <v>9000</v>
       </c>
       <c r="R14" s="1">
         <f t="shared" si="2"/>
-        <v>9300</v>
+        <v>9600</v>
       </c>
       <c r="S14" s="1">
         <f t="shared" si="2"/>
-        <v>9900</v>
+        <v>10200</v>
       </c>
       <c r="T14" s="1">
         <f t="shared" si="6"/>
-        <v>12900</v>
+        <v>13200</v>
       </c>
       <c r="U14" s="1">
         <f t="shared" si="3"/>
-        <v>13500</v>
+        <v>13800</v>
       </c>
       <c r="V14" s="2">
         <f t="shared" si="3"/>
-        <v>14100</v>
+        <v>14400</v>
       </c>
       <c r="W14" s="4">
         <f t="shared" si="2"/>
-        <v>14700</v>
+        <v>15000</v>
       </c>
       <c r="X14" s="3">
         <f t="shared" si="2"/>
-        <v>15900</v>
+        <v>16200</v>
       </c>
       <c r="Y14" s="1">
         <f t="shared" si="2"/>
-        <v>18900</v>
+        <v>19200</v>
       </c>
       <c r="Z14" s="1">
         <f t="shared" si="2"/>
-        <v>21900</v>
+        <v>22200</v>
       </c>
       <c r="AA14" s="9">
         <f t="shared" si="2"/>
-        <v>24900</v>
+        <v>25200</v>
       </c>
       <c r="AG14">
         <f t="shared" si="0"/>
@@ -2375,91 +2375,91 @@
       </c>
       <c r="F15" s="1">
         <f t="shared" si="5"/>
-        <v>1650</v>
+        <v>1980</v>
       </c>
       <c r="G15" s="1">
         <f t="shared" si="5"/>
-        <v>2310</v>
+        <v>2640</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="5"/>
-        <v>2970</v>
+        <v>3300</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="5"/>
-        <v>3630</v>
+        <v>3960</v>
       </c>
       <c r="J15" s="1">
         <f t="shared" si="2"/>
-        <v>4950</v>
+        <v>5280</v>
       </c>
       <c r="K15" s="1">
         <f t="shared" si="2"/>
-        <v>5610</v>
+        <v>5940</v>
       </c>
       <c r="L15" s="1">
         <f t="shared" si="2"/>
-        <v>6270</v>
+        <v>6600</v>
       </c>
       <c r="M15" s="1">
         <f t="shared" si="2"/>
-        <v>6930</v>
+        <v>7260</v>
       </c>
       <c r="N15" s="1">
         <f t="shared" si="2"/>
-        <v>7590</v>
+        <v>7920</v>
       </c>
       <c r="O15" s="1">
         <f t="shared" si="2"/>
-        <v>8250</v>
+        <v>8580</v>
       </c>
       <c r="P15" s="1">
         <f t="shared" si="2"/>
-        <v>8910</v>
+        <v>9240</v>
       </c>
       <c r="Q15" s="1">
         <f t="shared" si="2"/>
-        <v>9570</v>
+        <v>9900</v>
       </c>
       <c r="R15" s="1">
         <f t="shared" si="2"/>
-        <v>10230</v>
+        <v>10560</v>
       </c>
       <c r="S15" s="1">
         <f t="shared" si="2"/>
-        <v>10890</v>
+        <v>11220</v>
       </c>
       <c r="T15" s="1">
         <f t="shared" si="6"/>
-        <v>14190</v>
+        <v>14520</v>
       </c>
       <c r="U15" s="1">
         <f t="shared" si="3"/>
-        <v>14850</v>
+        <v>15180</v>
       </c>
       <c r="V15" s="2">
         <f t="shared" si="3"/>
-        <v>15510</v>
+        <v>15840</v>
       </c>
       <c r="W15" s="4">
         <f t="shared" si="2"/>
-        <v>16170</v>
+        <v>16500</v>
       </c>
       <c r="X15" s="3">
         <f t="shared" si="2"/>
-        <v>17490</v>
+        <v>17820</v>
       </c>
       <c r="Y15" s="1">
         <f t="shared" si="2"/>
-        <v>20790</v>
+        <v>21120</v>
       </c>
       <c r="Z15" s="1">
         <f t="shared" si="2"/>
-        <v>24090</v>
+        <v>24420</v>
       </c>
       <c r="AA15" s="9">
         <f t="shared" si="2"/>
-        <v>27390</v>
+        <v>27720</v>
       </c>
       <c r="AG15">
         <f t="shared" si="0"/>
@@ -2484,91 +2484,91 @@
       </c>
       <c r="F16" s="1">
         <f t="shared" si="5"/>
-        <v>1800</v>
+        <v>2160</v>
       </c>
       <c r="G16" s="1">
         <f t="shared" si="5"/>
-        <v>2520</v>
+        <v>2880</v>
       </c>
       <c r="H16" s="1">
         <f t="shared" si="5"/>
-        <v>3240</v>
+        <v>3600</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="5"/>
-        <v>3960</v>
+        <v>4320</v>
       </c>
       <c r="J16" s="1">
         <f t="shared" si="2"/>
-        <v>5400</v>
+        <v>5760</v>
       </c>
       <c r="K16" s="1">
         <f t="shared" si="2"/>
-        <v>6120</v>
+        <v>6480</v>
       </c>
       <c r="L16" s="1">
         <f t="shared" ref="J16:R21" si="8">$B$5*($D16+1)*(60/$B$3) + $B$4*($D16+1)*(60/$B$3) *L$4</f>
-        <v>6840</v>
+        <v>7200</v>
       </c>
       <c r="M16" s="1">
         <f t="shared" si="8"/>
-        <v>7560</v>
+        <v>7920</v>
       </c>
       <c r="N16" s="1">
         <f t="shared" si="8"/>
-        <v>8280</v>
+        <v>8640</v>
       </c>
       <c r="O16" s="1">
         <f t="shared" si="8"/>
-        <v>9000</v>
+        <v>9360</v>
       </c>
       <c r="P16" s="1">
         <f t="shared" si="8"/>
-        <v>9720</v>
+        <v>10080</v>
       </c>
       <c r="Q16" s="1">
         <f t="shared" si="8"/>
-        <v>10440</v>
+        <v>10800</v>
       </c>
       <c r="R16" s="1">
         <f t="shared" si="8"/>
-        <v>11160</v>
+        <v>11520</v>
       </c>
       <c r="S16" s="1">
         <f t="shared" si="2"/>
-        <v>11880</v>
+        <v>12240</v>
       </c>
       <c r="T16" s="1">
         <f t="shared" si="6"/>
-        <v>15480</v>
+        <v>15840</v>
       </c>
       <c r="U16" s="1">
         <f t="shared" si="3"/>
-        <v>16200</v>
+        <v>16560</v>
       </c>
       <c r="V16" s="2">
         <f t="shared" si="3"/>
-        <v>16920</v>
+        <v>17280</v>
       </c>
       <c r="W16" s="4">
         <f t="shared" si="2"/>
-        <v>17640</v>
+        <v>18000</v>
       </c>
       <c r="X16" s="3">
         <f t="shared" si="2"/>
-        <v>19080</v>
+        <v>19440</v>
       </c>
       <c r="Y16" s="1">
         <f t="shared" si="2"/>
-        <v>22680</v>
+        <v>23040</v>
       </c>
       <c r="Z16" s="1">
         <f t="shared" si="2"/>
-        <v>26280</v>
+        <v>26640</v>
       </c>
       <c r="AA16" s="9">
         <f t="shared" si="2"/>
-        <v>29880</v>
+        <v>30240</v>
       </c>
       <c r="AG16">
         <f t="shared" si="0"/>
@@ -2593,91 +2593,91 @@
       </c>
       <c r="F17" s="1">
         <f t="shared" si="5"/>
-        <v>1950</v>
+        <v>2340</v>
       </c>
       <c r="G17" s="1">
         <f t="shared" si="5"/>
-        <v>2730</v>
+        <v>3120</v>
       </c>
       <c r="H17" s="1">
         <f t="shared" si="5"/>
-        <v>3510</v>
+        <v>3900</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="5"/>
-        <v>4290</v>
+        <v>4680</v>
       </c>
       <c r="J17" s="1">
         <f t="shared" si="8"/>
-        <v>5850</v>
+        <v>6240</v>
       </c>
       <c r="K17" s="1">
         <f t="shared" si="8"/>
-        <v>6630</v>
+        <v>7020</v>
       </c>
       <c r="L17" s="1">
         <f t="shared" si="8"/>
-        <v>7410</v>
+        <v>7800</v>
       </c>
       <c r="M17" s="1">
         <f t="shared" si="8"/>
-        <v>8190</v>
+        <v>8580</v>
       </c>
       <c r="N17" s="1">
         <f t="shared" si="8"/>
-        <v>8970</v>
+        <v>9360</v>
       </c>
       <c r="O17" s="1">
         <f t="shared" si="8"/>
-        <v>9750</v>
+        <v>10140</v>
       </c>
       <c r="P17" s="1">
         <f t="shared" si="8"/>
-        <v>10530</v>
+        <v>10920</v>
       </c>
       <c r="Q17" s="1">
         <f t="shared" si="8"/>
-        <v>11310</v>
+        <v>11700</v>
       </c>
       <c r="R17" s="1">
         <f t="shared" si="8"/>
-        <v>12090</v>
+        <v>12480</v>
       </c>
       <c r="S17" s="1">
         <f t="shared" si="2"/>
-        <v>12870</v>
+        <v>13260</v>
       </c>
       <c r="T17" s="1">
         <f t="shared" si="6"/>
-        <v>16770</v>
+        <v>17160</v>
       </c>
       <c r="U17" s="1">
         <f t="shared" si="3"/>
-        <v>17550</v>
+        <v>17940</v>
       </c>
       <c r="V17" s="2">
         <f t="shared" si="3"/>
-        <v>18330</v>
+        <v>18720</v>
       </c>
       <c r="W17" s="4">
         <f t="shared" si="2"/>
-        <v>19110</v>
+        <v>19500</v>
       </c>
       <c r="X17" s="3">
         <f t="shared" si="2"/>
-        <v>20670</v>
+        <v>21060</v>
       </c>
       <c r="Y17" s="1">
         <f t="shared" si="2"/>
-        <v>24570</v>
+        <v>24960</v>
       </c>
       <c r="Z17" s="1">
         <f t="shared" si="2"/>
-        <v>28470</v>
+        <v>28860</v>
       </c>
       <c r="AA17" s="9">
         <f t="shared" si="2"/>
-        <v>32370</v>
+        <v>32760</v>
       </c>
       <c r="AG17">
         <f t="shared" si="0"/>
@@ -2702,91 +2702,91 @@
       </c>
       <c r="F18" s="1">
         <f t="shared" si="5"/>
-        <v>2100</v>
+        <v>2520</v>
       </c>
       <c r="G18" s="1">
         <f t="shared" si="5"/>
-        <v>2940</v>
+        <v>3360</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="5"/>
-        <v>3780</v>
+        <v>4200</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="5"/>
-        <v>4620</v>
+        <v>5040</v>
       </c>
       <c r="J18" s="1">
         <f t="shared" si="8"/>
-        <v>6300</v>
+        <v>6720</v>
       </c>
       <c r="K18" s="1">
         <f t="shared" si="8"/>
-        <v>7140</v>
+        <v>7560</v>
       </c>
       <c r="L18" s="1">
         <f t="shared" si="8"/>
-        <v>7980</v>
+        <v>8400</v>
       </c>
       <c r="M18" s="1">
         <f t="shared" si="8"/>
-        <v>8820</v>
+        <v>9240</v>
       </c>
       <c r="N18" s="1">
         <f t="shared" si="8"/>
-        <v>9660</v>
+        <v>10080</v>
       </c>
       <c r="O18" s="1">
         <f t="shared" si="8"/>
-        <v>10500</v>
+        <v>10920</v>
       </c>
       <c r="P18" s="1">
         <f t="shared" si="8"/>
-        <v>11340</v>
+        <v>11760</v>
       </c>
       <c r="Q18" s="1">
         <f t="shared" si="8"/>
-        <v>12180</v>
+        <v>12600</v>
       </c>
       <c r="R18" s="1">
         <f t="shared" si="8"/>
-        <v>13020</v>
+        <v>13440</v>
       </c>
       <c r="S18" s="1">
         <f t="shared" si="2"/>
-        <v>13860</v>
+        <v>14280</v>
       </c>
       <c r="T18" s="1">
         <f t="shared" si="6"/>
-        <v>18060</v>
+        <v>18480</v>
       </c>
       <c r="U18" s="1">
         <f t="shared" si="3"/>
-        <v>18900</v>
+        <v>19320</v>
       </c>
       <c r="V18" s="2">
         <f t="shared" si="3"/>
-        <v>19740</v>
+        <v>20160</v>
       </c>
       <c r="W18" s="4">
         <f t="shared" si="2"/>
-        <v>20580</v>
+        <v>21000</v>
       </c>
       <c r="X18" s="3">
         <f t="shared" si="2"/>
-        <v>22260</v>
+        <v>22680</v>
       </c>
       <c r="Y18" s="1">
         <f t="shared" si="2"/>
-        <v>26460</v>
+        <v>26880</v>
       </c>
       <c r="Z18" s="1">
         <f t="shared" si="2"/>
-        <v>30660</v>
+        <v>31080</v>
       </c>
       <c r="AA18" s="9">
         <f t="shared" si="2"/>
-        <v>34860</v>
+        <v>35280</v>
       </c>
       <c r="AG18">
         <f t="shared" si="0"/>
@@ -2811,91 +2811,91 @@
       </c>
       <c r="F19" s="1">
         <f t="shared" si="5"/>
-        <v>2250</v>
+        <v>2700</v>
       </c>
       <c r="G19" s="1">
         <f t="shared" si="5"/>
-        <v>3150</v>
+        <v>3600</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="5"/>
-        <v>4050</v>
+        <v>4500</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" si="5"/>
-        <v>4950</v>
+        <v>5400</v>
       </c>
       <c r="J19" s="1">
         <f t="shared" si="8"/>
-        <v>6750</v>
+        <v>7200</v>
       </c>
       <c r="K19" s="1">
         <f t="shared" si="8"/>
-        <v>7650</v>
+        <v>8100</v>
       </c>
       <c r="L19" s="1">
         <f t="shared" si="8"/>
-        <v>8550</v>
+        <v>9000</v>
       </c>
       <c r="M19" s="1">
         <f t="shared" si="8"/>
-        <v>9450</v>
+        <v>9900</v>
       </c>
       <c r="N19" s="1">
         <f t="shared" si="8"/>
-        <v>10350</v>
+        <v>10800</v>
       </c>
       <c r="O19" s="1">
         <f t="shared" si="8"/>
-        <v>11250</v>
+        <v>11700</v>
       </c>
       <c r="P19" s="1">
         <f t="shared" si="8"/>
-        <v>12150</v>
+        <v>12600</v>
       </c>
       <c r="Q19" s="1">
         <f t="shared" si="8"/>
-        <v>13050</v>
+        <v>13500</v>
       </c>
       <c r="R19" s="1">
         <f t="shared" si="8"/>
-        <v>13950</v>
+        <v>14400</v>
       </c>
       <c r="S19" s="1">
         <f t="shared" si="2"/>
-        <v>14850</v>
+        <v>15300</v>
       </c>
       <c r="T19" s="1">
         <f t="shared" si="6"/>
-        <v>19350</v>
+        <v>19800</v>
       </c>
       <c r="U19" s="1">
         <f t="shared" si="3"/>
-        <v>20250</v>
+        <v>20700</v>
       </c>
       <c r="V19" s="2">
         <f t="shared" si="3"/>
-        <v>21150</v>
+        <v>21600</v>
       </c>
       <c r="W19" s="4">
         <f t="shared" si="2"/>
-        <v>22050</v>
+        <v>22500</v>
       </c>
       <c r="X19" s="3">
         <f t="shared" si="2"/>
-        <v>23850</v>
+        <v>24300</v>
       </c>
       <c r="Y19" s="1">
         <f t="shared" si="2"/>
-        <v>28350</v>
+        <v>28800</v>
       </c>
       <c r="Z19" s="1">
         <f t="shared" si="2"/>
-        <v>32850</v>
+        <v>33300</v>
       </c>
       <c r="AA19" s="9">
         <f t="shared" si="2"/>
-        <v>37350</v>
+        <v>37800</v>
       </c>
       <c r="AG19">
         <f t="shared" si="0"/>
@@ -2920,91 +2920,91 @@
       </c>
       <c r="F20" s="1">
         <f t="shared" si="5"/>
-        <v>2400</v>
+        <v>2880</v>
       </c>
       <c r="G20" s="1">
         <f t="shared" si="5"/>
-        <v>3360</v>
+        <v>3840</v>
       </c>
       <c r="H20" s="1">
         <f t="shared" si="5"/>
-        <v>4320</v>
+        <v>4800</v>
       </c>
       <c r="I20" s="1">
         <f t="shared" si="5"/>
-        <v>5280</v>
+        <v>5760</v>
       </c>
       <c r="J20" s="1">
         <f t="shared" si="8"/>
-        <v>7200</v>
+        <v>7680</v>
       </c>
       <c r="K20" s="1">
         <f t="shared" si="8"/>
-        <v>8160</v>
+        <v>8640</v>
       </c>
       <c r="L20" s="1">
         <f t="shared" si="8"/>
-        <v>9120</v>
+        <v>9600</v>
       </c>
       <c r="M20" s="1">
         <f t="shared" si="8"/>
-        <v>10080</v>
+        <v>10560</v>
       </c>
       <c r="N20" s="1">
         <f t="shared" si="8"/>
-        <v>11040</v>
+        <v>11520</v>
       </c>
       <c r="O20" s="1">
         <f t="shared" si="8"/>
-        <v>12000</v>
+        <v>12480</v>
       </c>
       <c r="P20" s="1">
         <f t="shared" si="8"/>
-        <v>12960</v>
+        <v>13440</v>
       </c>
       <c r="Q20" s="1">
         <f t="shared" si="8"/>
-        <v>13920</v>
+        <v>14400</v>
       </c>
       <c r="R20" s="1">
         <f t="shared" si="8"/>
-        <v>14880</v>
+        <v>15360</v>
       </c>
       <c r="S20" s="1">
         <f t="shared" si="2"/>
-        <v>15840</v>
+        <v>16320</v>
       </c>
       <c r="T20" s="1">
         <f t="shared" si="6"/>
-        <v>20640</v>
+        <v>21120</v>
       </c>
       <c r="U20" s="1">
         <f t="shared" si="3"/>
-        <v>21600</v>
+        <v>22080</v>
       </c>
       <c r="V20" s="2">
         <f t="shared" si="3"/>
-        <v>22560</v>
+        <v>23040</v>
       </c>
       <c r="W20" s="4">
         <f t="shared" si="2"/>
-        <v>23520</v>
+        <v>24000</v>
       </c>
       <c r="X20" s="3">
         <f t="shared" si="2"/>
-        <v>25440</v>
+        <v>25920</v>
       </c>
       <c r="Y20" s="1">
         <f t="shared" si="2"/>
-        <v>30240</v>
+        <v>30720</v>
       </c>
       <c r="Z20" s="1">
         <f t="shared" si="2"/>
-        <v>35040</v>
+        <v>35520</v>
       </c>
       <c r="AA20" s="9">
         <f t="shared" si="2"/>
-        <v>39840</v>
+        <v>40320</v>
       </c>
       <c r="AG20">
         <f t="shared" si="0"/>
@@ -3029,91 +3029,91 @@
       </c>
       <c r="F21" s="1">
         <f t="shared" si="5"/>
-        <v>2550</v>
+        <v>3060</v>
       </c>
       <c r="G21" s="1">
         <f t="shared" si="5"/>
-        <v>3570</v>
+        <v>4080</v>
       </c>
       <c r="H21" s="1">
         <f t="shared" si="5"/>
-        <v>4590</v>
+        <v>5100</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="5"/>
-        <v>5610</v>
+        <v>6120</v>
       </c>
       <c r="J21" s="1">
         <f t="shared" si="8"/>
-        <v>7650</v>
+        <v>8160</v>
       </c>
       <c r="K21" s="1">
         <f t="shared" si="8"/>
-        <v>8670</v>
+        <v>9180</v>
       </c>
       <c r="L21" s="1">
         <f t="shared" si="8"/>
-        <v>9690</v>
+        <v>10200</v>
       </c>
       <c r="M21" s="1">
         <f t="shared" si="8"/>
-        <v>10710</v>
+        <v>11220</v>
       </c>
       <c r="N21" s="1">
         <f t="shared" si="8"/>
-        <v>11730</v>
+        <v>12240</v>
       </c>
       <c r="O21" s="1">
         <f t="shared" si="8"/>
-        <v>12750</v>
+        <v>13260</v>
       </c>
       <c r="P21" s="1">
         <f t="shared" si="8"/>
-        <v>13770</v>
+        <v>14280</v>
       </c>
       <c r="Q21" s="1">
         <f t="shared" si="8"/>
-        <v>14790</v>
+        <v>15300</v>
       </c>
       <c r="R21" s="1">
         <f t="shared" si="8"/>
-        <v>15810</v>
+        <v>16320</v>
       </c>
       <c r="S21" s="1">
         <f t="shared" si="5"/>
-        <v>16830</v>
+        <v>17340</v>
       </c>
       <c r="T21" s="1">
         <f t="shared" si="6"/>
-        <v>21930</v>
+        <v>22440</v>
       </c>
       <c r="U21" s="1">
         <f t="shared" si="6"/>
-        <v>22950</v>
+        <v>23460</v>
       </c>
       <c r="V21" s="2">
         <f t="shared" si="6"/>
-        <v>23970</v>
+        <v>24480</v>
       </c>
       <c r="W21" s="4">
         <f t="shared" si="5"/>
-        <v>24990</v>
+        <v>25500</v>
       </c>
       <c r="X21" s="3">
         <f t="shared" si="5"/>
-        <v>27030</v>
+        <v>27540</v>
       </c>
       <c r="Y21" s="1">
         <f t="shared" si="5"/>
-        <v>32130</v>
+        <v>32640</v>
       </c>
       <c r="Z21" s="1">
         <f t="shared" si="5"/>
-        <v>37230</v>
+        <v>37740</v>
       </c>
       <c r="AA21" s="9">
         <f t="shared" si="5"/>
-        <v>42330</v>
+        <v>42840</v>
       </c>
       <c r="AG21">
         <f t="shared" si="0"/>
@@ -3138,91 +3138,91 @@
       </c>
       <c r="F22" s="16">
         <f t="shared" si="5"/>
-        <v>2700</v>
+        <v>3240</v>
       </c>
       <c r="G22" s="16">
         <f t="shared" si="5"/>
-        <v>3780</v>
+        <v>4320</v>
       </c>
       <c r="H22" s="16">
         <f t="shared" si="5"/>
-        <v>4860</v>
+        <v>5400</v>
       </c>
       <c r="I22" s="16">
         <f t="shared" si="5"/>
-        <v>5940</v>
+        <v>6480</v>
       </c>
       <c r="J22" s="16">
         <f t="shared" si="5"/>
-        <v>8100</v>
+        <v>8640</v>
       </c>
       <c r="K22" s="16">
         <f t="shared" si="5"/>
-        <v>9180</v>
+        <v>9720</v>
       </c>
       <c r="L22" s="16">
         <f t="shared" si="5"/>
-        <v>10260</v>
+        <v>10800</v>
       </c>
       <c r="M22" s="16">
         <f t="shared" si="5"/>
-        <v>11340</v>
+        <v>11880</v>
       </c>
       <c r="N22" s="16">
         <f t="shared" si="5"/>
-        <v>12420</v>
+        <v>12960</v>
       </c>
       <c r="O22" s="16">
         <f t="shared" si="5"/>
-        <v>13500</v>
+        <v>14040</v>
       </c>
       <c r="P22" s="16">
         <f t="shared" si="5"/>
-        <v>14580</v>
+        <v>15120</v>
       </c>
       <c r="Q22" s="16">
         <f t="shared" si="5"/>
-        <v>15660</v>
+        <v>16200</v>
       </c>
       <c r="R22" s="16">
         <f t="shared" si="5"/>
-        <v>16740</v>
+        <v>17280</v>
       </c>
       <c r="S22" s="16">
         <f t="shared" si="5"/>
-        <v>17820</v>
+        <v>18360</v>
       </c>
       <c r="T22" s="16">
         <f t="shared" si="6"/>
-        <v>23220</v>
+        <v>23760</v>
       </c>
       <c r="U22" s="16">
         <f t="shared" si="6"/>
-        <v>24300</v>
+        <v>24840</v>
       </c>
       <c r="V22" s="17">
         <f t="shared" si="6"/>
-        <v>25380</v>
+        <v>25920</v>
       </c>
       <c r="W22" s="5">
         <f t="shared" si="5"/>
-        <v>26460</v>
+        <v>27000</v>
       </c>
       <c r="X22" s="19">
         <f t="shared" si="5"/>
-        <v>28620</v>
+        <v>29160</v>
       </c>
       <c r="Y22" s="16">
         <f t="shared" si="5"/>
-        <v>34020</v>
+        <v>34560</v>
       </c>
       <c r="Z22" s="16">
         <f t="shared" si="5"/>
-        <v>39420</v>
+        <v>39960</v>
       </c>
       <c r="AA22" s="11">
         <f t="shared" si="5"/>
-        <v>44820</v>
+        <v>45360</v>
       </c>
       <c r="AG22">
         <f t="shared" si="0"/>
@@ -3247,91 +3247,91 @@
       </c>
       <c r="F23" s="12">
         <f t="shared" si="5"/>
-        <v>2850</v>
+        <v>3420</v>
       </c>
       <c r="G23" s="12">
         <f t="shared" si="5"/>
-        <v>3990</v>
+        <v>4560</v>
       </c>
       <c r="H23" s="12">
         <f t="shared" si="5"/>
-        <v>5130</v>
+        <v>5700</v>
       </c>
       <c r="I23" s="12">
         <f t="shared" si="5"/>
-        <v>6270</v>
+        <v>6840</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="5"/>
-        <v>8550</v>
+        <v>9120</v>
       </c>
       <c r="K23" s="12">
         <f t="shared" si="5"/>
-        <v>9690</v>
+        <v>10260</v>
       </c>
       <c r="L23" s="12">
         <f t="shared" si="5"/>
-        <v>10830</v>
+        <v>11400</v>
       </c>
       <c r="M23" s="12">
         <f t="shared" si="5"/>
-        <v>11970</v>
+        <v>12540</v>
       </c>
       <c r="N23" s="12">
         <f t="shared" si="5"/>
-        <v>13110</v>
+        <v>13680</v>
       </c>
       <c r="O23" s="12">
         <f t="shared" si="5"/>
-        <v>14250</v>
+        <v>14820</v>
       </c>
       <c r="P23" s="12">
         <f t="shared" si="5"/>
-        <v>15390</v>
+        <v>15960</v>
       </c>
       <c r="Q23" s="12">
         <f t="shared" si="5"/>
-        <v>16530</v>
+        <v>17100</v>
       </c>
       <c r="R23" s="12">
         <f t="shared" si="5"/>
-        <v>17670</v>
+        <v>18240</v>
       </c>
       <c r="S23" s="12">
         <f t="shared" si="5"/>
-        <v>18810</v>
+        <v>19380</v>
       </c>
       <c r="T23" s="12">
         <f t="shared" si="6"/>
-        <v>24510</v>
+        <v>25080</v>
       </c>
       <c r="U23" s="12">
         <f t="shared" si="6"/>
-        <v>25650</v>
+        <v>26220</v>
       </c>
       <c r="V23" s="13">
         <f t="shared" si="6"/>
-        <v>26790</v>
+        <v>27360</v>
       </c>
       <c r="W23" s="14">
         <f t="shared" si="5"/>
-        <v>27930</v>
+        <v>28500</v>
       </c>
       <c r="X23" s="15">
         <f t="shared" si="5"/>
-        <v>30210</v>
+        <v>30780</v>
       </c>
       <c r="Y23" s="12">
         <f t="shared" si="5"/>
-        <v>35910</v>
+        <v>36480</v>
       </c>
       <c r="Z23" s="12">
         <f t="shared" si="5"/>
-        <v>41610</v>
+        <v>42180</v>
       </c>
       <c r="AA23" s="25">
         <f t="shared" si="5"/>
-        <v>47310</v>
+        <v>47880</v>
       </c>
       <c r="AG23">
         <f t="shared" si="0"/>
@@ -3356,91 +3356,91 @@
       </c>
       <c r="F24" s="1">
         <f t="shared" si="5"/>
-        <v>3000</v>
+        <v>3600</v>
       </c>
       <c r="G24" s="1">
         <f t="shared" si="5"/>
-        <v>4200</v>
+        <v>4800</v>
       </c>
       <c r="H24" s="1">
         <f t="shared" si="5"/>
-        <v>5400</v>
+        <v>6000</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" si="5"/>
-        <v>6600</v>
+        <v>7200</v>
       </c>
       <c r="J24" s="1">
         <f t="shared" si="5"/>
-        <v>9000</v>
+        <v>9600</v>
       </c>
       <c r="K24" s="1">
         <f t="shared" si="5"/>
-        <v>10200</v>
+        <v>10800</v>
       </c>
       <c r="L24" s="1">
         <f t="shared" si="5"/>
-        <v>11400</v>
+        <v>12000</v>
       </c>
       <c r="M24" s="1">
         <f t="shared" si="5"/>
-        <v>12600</v>
+        <v>13200</v>
       </c>
       <c r="N24" s="1">
         <f t="shared" si="5"/>
-        <v>13800</v>
+        <v>14400</v>
       </c>
       <c r="O24" s="1">
         <f t="shared" si="5"/>
-        <v>15000</v>
+        <v>15600</v>
       </c>
       <c r="P24" s="1">
         <f t="shared" si="5"/>
-        <v>16200</v>
+        <v>16800</v>
       </c>
       <c r="Q24" s="1">
         <f t="shared" si="5"/>
-        <v>17400</v>
+        <v>18000</v>
       </c>
       <c r="R24" s="1">
         <f t="shared" si="5"/>
-        <v>18600</v>
+        <v>19200</v>
       </c>
       <c r="S24" s="1">
         <f t="shared" si="5"/>
-        <v>19800</v>
+        <v>20400</v>
       </c>
       <c r="T24" s="1">
         <f t="shared" si="6"/>
-        <v>25800</v>
+        <v>26400</v>
       </c>
       <c r="U24" s="1">
         <f t="shared" si="6"/>
-        <v>27000</v>
+        <v>27600</v>
       </c>
       <c r="V24" s="2">
         <f t="shared" si="6"/>
-        <v>28200</v>
+        <v>28800</v>
       </c>
       <c r="W24" s="4">
         <f t="shared" si="5"/>
-        <v>29400</v>
+        <v>30000</v>
       </c>
       <c r="X24" s="3">
         <f t="shared" si="5"/>
-        <v>31800</v>
+        <v>32400</v>
       </c>
       <c r="Y24" s="1">
         <f t="shared" si="5"/>
-        <v>37800</v>
+        <v>38400</v>
       </c>
       <c r="Z24" s="1">
         <f t="shared" si="5"/>
-        <v>43800</v>
+        <v>44400</v>
       </c>
       <c r="AA24" s="9">
         <f t="shared" si="5"/>
-        <v>49800</v>
+        <v>50400</v>
       </c>
       <c r="AG24">
         <f t="shared" si="0"/>
@@ -3465,91 +3465,91 @@
       </c>
       <c r="F25" s="1">
         <f t="shared" si="5"/>
-        <v>3150</v>
+        <v>3780</v>
       </c>
       <c r="G25" s="1">
         <f t="shared" si="5"/>
-        <v>4410</v>
+        <v>5040</v>
       </c>
       <c r="H25" s="1">
         <f t="shared" si="5"/>
-        <v>5670</v>
+        <v>6300</v>
       </c>
       <c r="I25" s="1">
         <f t="shared" si="5"/>
-        <v>6930</v>
+        <v>7560</v>
       </c>
       <c r="J25" s="1">
         <f t="shared" si="5"/>
-        <v>9450</v>
+        <v>10080</v>
       </c>
       <c r="K25" s="1">
         <f t="shared" si="5"/>
-        <v>10710</v>
+        <v>11340</v>
       </c>
       <c r="L25" s="1">
         <f t="shared" si="5"/>
-        <v>11970</v>
+        <v>12600</v>
       </c>
       <c r="M25" s="1">
         <f t="shared" si="5"/>
-        <v>13230</v>
+        <v>13860</v>
       </c>
       <c r="N25" s="1">
         <f t="shared" si="5"/>
-        <v>14490</v>
+        <v>15120</v>
       </c>
       <c r="O25" s="1">
         <f t="shared" si="5"/>
-        <v>15750</v>
+        <v>16380</v>
       </c>
       <c r="P25" s="1">
         <f t="shared" si="5"/>
-        <v>17010</v>
+        <v>17640</v>
       </c>
       <c r="Q25" s="1">
         <f t="shared" si="5"/>
-        <v>18270</v>
+        <v>18900</v>
       </c>
       <c r="R25" s="1">
         <f t="shared" si="5"/>
-        <v>19530</v>
+        <v>20160</v>
       </c>
       <c r="S25" s="1">
         <f t="shared" si="5"/>
-        <v>20790</v>
+        <v>21420</v>
       </c>
       <c r="T25" s="1">
         <f t="shared" si="6"/>
-        <v>27090</v>
+        <v>27720</v>
       </c>
       <c r="U25" s="1">
         <f t="shared" si="6"/>
-        <v>28350</v>
+        <v>28980</v>
       </c>
       <c r="V25" s="2">
         <f t="shared" si="6"/>
-        <v>29610</v>
+        <v>30240</v>
       </c>
       <c r="W25" s="4">
         <f t="shared" si="5"/>
-        <v>30870</v>
+        <v>31500</v>
       </c>
       <c r="X25" s="3">
         <f t="shared" si="5"/>
-        <v>33390</v>
+        <v>34020</v>
       </c>
       <c r="Y25" s="1">
         <f t="shared" si="5"/>
-        <v>39690</v>
+        <v>40320</v>
       </c>
       <c r="Z25" s="1">
         <f t="shared" si="5"/>
-        <v>45990</v>
+        <v>46620</v>
       </c>
       <c r="AA25" s="9">
         <f t="shared" si="5"/>
-        <v>52290</v>
+        <v>52920</v>
       </c>
       <c r="AG25">
         <f t="shared" si="0"/>
@@ -3574,91 +3574,91 @@
       </c>
       <c r="F26" s="1">
         <f t="shared" si="5"/>
-        <v>3300</v>
+        <v>3960</v>
       </c>
       <c r="G26" s="1">
         <f t="shared" si="5"/>
-        <v>4620</v>
+        <v>5280</v>
       </c>
       <c r="H26" s="1">
         <f t="shared" si="5"/>
-        <v>5940</v>
+        <v>6600</v>
       </c>
       <c r="I26" s="1">
         <f t="shared" si="5"/>
-        <v>7260</v>
+        <v>7920</v>
       </c>
       <c r="J26" s="1">
         <f t="shared" si="5"/>
-        <v>9900</v>
+        <v>10560</v>
       </c>
       <c r="K26" s="1">
         <f t="shared" si="5"/>
-        <v>11220</v>
+        <v>11880</v>
       </c>
       <c r="L26" s="1">
         <f t="shared" si="5"/>
-        <v>12540</v>
+        <v>13200</v>
       </c>
       <c r="M26" s="1">
         <f t="shared" si="5"/>
-        <v>13860</v>
+        <v>14520</v>
       </c>
       <c r="N26" s="1">
         <f t="shared" si="5"/>
-        <v>15180</v>
+        <v>15840</v>
       </c>
       <c r="O26" s="1">
         <f t="shared" si="5"/>
-        <v>16500</v>
+        <v>17160</v>
       </c>
       <c r="P26" s="1">
         <f t="shared" si="5"/>
-        <v>17820</v>
+        <v>18480</v>
       </c>
       <c r="Q26" s="1">
         <f t="shared" si="5"/>
-        <v>19140</v>
+        <v>19800</v>
       </c>
       <c r="R26" s="1">
         <f t="shared" si="5"/>
-        <v>20460</v>
+        <v>21120</v>
       </c>
       <c r="S26" s="1">
         <f t="shared" si="5"/>
-        <v>21780</v>
+        <v>22440</v>
       </c>
       <c r="T26" s="1">
         <f t="shared" si="6"/>
-        <v>28380</v>
+        <v>29040</v>
       </c>
       <c r="U26" s="1">
         <f t="shared" si="6"/>
-        <v>29700</v>
+        <v>30360</v>
       </c>
       <c r="V26" s="2">
         <f t="shared" si="6"/>
-        <v>31020</v>
+        <v>31680</v>
       </c>
       <c r="W26" s="4">
         <f t="shared" si="5"/>
-        <v>32340</v>
+        <v>33000</v>
       </c>
       <c r="X26" s="3">
         <f t="shared" si="5"/>
-        <v>34980</v>
+        <v>35640</v>
       </c>
       <c r="Y26" s="1">
         <f t="shared" si="5"/>
-        <v>41580</v>
+        <v>42240</v>
       </c>
       <c r="Z26" s="1">
         <f t="shared" si="5"/>
-        <v>48180</v>
+        <v>48840</v>
       </c>
       <c r="AA26" s="9">
         <f t="shared" si="5"/>
-        <v>54780</v>
+        <v>55440</v>
       </c>
       <c r="AG26">
         <f t="shared" si="0"/>
@@ -3683,91 +3683,91 @@
       </c>
       <c r="F27" s="1">
         <f t="shared" si="5"/>
-        <v>3450</v>
+        <v>4140</v>
       </c>
       <c r="G27" s="1">
         <f t="shared" si="5"/>
-        <v>4830</v>
+        <v>5520</v>
       </c>
       <c r="H27" s="1">
         <f t="shared" si="5"/>
-        <v>6210</v>
+        <v>6900</v>
       </c>
       <c r="I27" s="1">
         <f t="shared" si="5"/>
-        <v>7590</v>
+        <v>8280</v>
       </c>
       <c r="J27" s="1">
         <f t="shared" si="5"/>
-        <v>10350</v>
+        <v>11040</v>
       </c>
       <c r="K27" s="1">
         <f t="shared" si="5"/>
-        <v>11730</v>
+        <v>12420</v>
       </c>
       <c r="L27" s="1">
         <f t="shared" si="5"/>
-        <v>13110</v>
+        <v>13800</v>
       </c>
       <c r="M27" s="1">
         <f t="shared" si="5"/>
-        <v>14490</v>
+        <v>15180</v>
       </c>
       <c r="N27" s="1">
         <f t="shared" si="5"/>
-        <v>15870</v>
+        <v>16560</v>
       </c>
       <c r="O27" s="1">
         <f t="shared" si="5"/>
-        <v>17250</v>
+        <v>17940</v>
       </c>
       <c r="P27" s="1">
         <f t="shared" si="5"/>
-        <v>18630</v>
+        <v>19320</v>
       </c>
       <c r="Q27" s="1">
         <f t="shared" si="5"/>
-        <v>20010</v>
+        <v>20700</v>
       </c>
       <c r="R27" s="1">
         <f t="shared" si="5"/>
-        <v>21390</v>
+        <v>22080</v>
       </c>
       <c r="S27" s="1">
         <f t="shared" si="5"/>
-        <v>22770</v>
+        <v>23460</v>
       </c>
       <c r="T27" s="1">
         <f t="shared" si="6"/>
-        <v>29670</v>
+        <v>30360</v>
       </c>
       <c r="U27" s="1">
         <f t="shared" si="6"/>
-        <v>31050</v>
+        <v>31740</v>
       </c>
       <c r="V27" s="2">
         <f t="shared" si="6"/>
-        <v>32430</v>
+        <v>33120</v>
       </c>
       <c r="W27" s="4">
         <f t="shared" si="5"/>
-        <v>33810</v>
+        <v>34500</v>
       </c>
       <c r="X27" s="3">
         <f t="shared" si="5"/>
-        <v>36570</v>
+        <v>37260</v>
       </c>
       <c r="Y27" s="1">
         <f t="shared" si="5"/>
-        <v>43470</v>
+        <v>44160</v>
       </c>
       <c r="Z27" s="1">
         <f t="shared" si="5"/>
-        <v>50370</v>
+        <v>51060</v>
       </c>
       <c r="AA27" s="9">
         <f t="shared" si="5"/>
-        <v>57270</v>
+        <v>57960</v>
       </c>
       <c r="AG27">
         <f t="shared" si="0"/>
@@ -3792,91 +3792,91 @@
       </c>
       <c r="F28" s="16">
         <f t="shared" si="5"/>
-        <v>3600</v>
+        <v>4320</v>
       </c>
       <c r="G28" s="16">
         <f t="shared" si="5"/>
-        <v>5040</v>
+        <v>5760</v>
       </c>
       <c r="H28" s="16">
         <f t="shared" si="5"/>
-        <v>6480</v>
+        <v>7200</v>
       </c>
       <c r="I28" s="16">
         <f t="shared" si="5"/>
-        <v>7920</v>
+        <v>8640</v>
       </c>
       <c r="J28" s="16">
         <f t="shared" si="5"/>
-        <v>10800</v>
+        <v>11520</v>
       </c>
       <c r="K28" s="16">
         <f t="shared" si="5"/>
-        <v>12240</v>
+        <v>12960</v>
       </c>
       <c r="L28" s="16">
         <f t="shared" si="5"/>
-        <v>13680</v>
+        <v>14400</v>
       </c>
       <c r="M28" s="16">
         <f t="shared" si="5"/>
-        <v>15120</v>
+        <v>15840</v>
       </c>
       <c r="N28" s="16">
         <f t="shared" si="5"/>
-        <v>16560</v>
+        <v>17280</v>
       </c>
       <c r="O28" s="16">
         <f t="shared" si="5"/>
-        <v>18000</v>
+        <v>18720</v>
       </c>
       <c r="P28" s="16">
         <f t="shared" si="5"/>
-        <v>19440</v>
+        <v>20160</v>
       </c>
       <c r="Q28" s="16">
         <f t="shared" si="5"/>
-        <v>20880</v>
+        <v>21600</v>
       </c>
       <c r="R28" s="16">
         <f t="shared" si="5"/>
-        <v>22320</v>
+        <v>23040</v>
       </c>
       <c r="S28" s="16">
         <f t="shared" si="5"/>
-        <v>23760</v>
+        <v>24480</v>
       </c>
       <c r="T28" s="16">
         <f t="shared" si="6"/>
-        <v>30960</v>
+        <v>31680</v>
       </c>
       <c r="U28" s="16">
         <f t="shared" si="6"/>
-        <v>32400</v>
+        <v>33120</v>
       </c>
       <c r="V28" s="17">
         <f t="shared" si="6"/>
-        <v>33840</v>
+        <v>34560</v>
       </c>
       <c r="W28" s="5">
         <f t="shared" si="5"/>
-        <v>35280</v>
+        <v>36000</v>
       </c>
       <c r="X28" s="19">
         <f t="shared" si="5"/>
-        <v>38160</v>
+        <v>38880</v>
       </c>
       <c r="Y28" s="16">
         <f t="shared" si="5"/>
-        <v>45360</v>
+        <v>46080</v>
       </c>
       <c r="Z28" s="16">
         <f t="shared" si="5"/>
-        <v>52560</v>
+        <v>53280</v>
       </c>
       <c r="AA28" s="11">
         <f t="shared" si="5"/>
-        <v>59760</v>
+        <v>60480</v>
       </c>
       <c r="AG28">
         <f t="shared" si="0"/>

</xml_diff>